<commit_message>
Leave Application Foundation Done
</commit_message>
<xml_diff>
--- a/leave application/CS Form No. 6, Revised 2020 (Application for Leave) (Fillable).xlsx
+++ b/leave application/CS Form No. 6, Revised 2020 (Application for Leave) (Fillable).xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bless\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bless\Music\boac-personnel-hub\leave application\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6141A02-CDFF-4A88-AD09-0FD43DBAC715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DDFB5F-8EF8-4A03-B2FA-3A15835B02B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
   <si>
     <t>APPLICATION FOR LEAVE</t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>_____________________________________________</t>
-  </si>
-  <si>
-    <t>________________________________________</t>
   </si>
   <si>
     <t>_______ days with pay</t>
@@ -175,9 +172,6 @@
   </si>
   <si>
     <t xml:space="preserve">Others: </t>
-  </si>
-  <si>
-    <t>_____________________________________</t>
   </si>
   <si>
     <r>
@@ -550,7 +544,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -811,11 +805,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -863,9 +868,6 @@
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -953,7 +955,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -972,6 +977,19 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3044,1914 +3062,6 @@
     </mc:Choice>
     <mc:Fallback/>
   </mc:AlternateContent>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>658812</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>63501</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>2952750</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>261938</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3317875" y="1952626"/>
-          <a:ext cx="4095750" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1"/>
-            <a:t>DELA CRUZ,</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t> JUAN D.</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>952501</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1103312</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>261937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="TextBox 38">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000027000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1254126" y="2278063"/>
-          <a:ext cx="1349374" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1"/>
-            <a:t>April</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t> 17, 2021</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>817563</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1135063</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>246062</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="TextBox 39">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000028000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3476626" y="2262188"/>
-          <a:ext cx="2119312" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1"/>
-            <a:t>Administrative</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t> Assistant I</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>2024063</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>79375</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032125</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>277812</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="41" name="TextBox 40">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000029000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6484938" y="2293938"/>
-          <a:ext cx="1008062" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>₱ 0.00</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1246187</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>174624</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032124</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>134936</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="TextBox 41">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5707062" y="3452812"/>
-          <a:ext cx="1785937" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>Residence</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1000125</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032125</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>134937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="TextBox 42">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002B000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5461000" y="3690938"/>
-          <a:ext cx="2032000" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1539875</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>166688</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3016250</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="TextBox 43">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002C000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6000750" y="4159251"/>
-          <a:ext cx="1476375" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1571625</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>7937</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3016250</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="TextBox 44">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002D000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6032500" y="4413250"/>
-          <a:ext cx="1444625" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>7937</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>7937</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3024188</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="TextBox 45">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4294187" y="4651375"/>
-          <a:ext cx="3190876" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>738187</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>2984500</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>134937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="TextBox 46">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00002F000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5199062" y="5119688"/>
-          <a:ext cx="2246313" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>23812</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>7937</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3016250</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="48" name="TextBox 47">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000030000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4310062" y="5365750"/>
-          <a:ext cx="3167063" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>31750</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>166688</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>119062</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="49" name="TextBox 48">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000031000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="158750" y="6786563"/>
-          <a:ext cx="2619375" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>150812</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>7938</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>7937</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="TextBox 49">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000032000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="277812" y="7350126"/>
-          <a:ext cx="1230313" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>2 days</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>198437</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="51" name="TextBox 50">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000033000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="301625" y="7818438"/>
-          <a:ext cx="1817688" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>April 28-29, 2021</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1016001</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>7938</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>150812</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="52" name="TextBox 51">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000034000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1317626" y="8850313"/>
-          <a:ext cx="1785937" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>March 2021</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>1309688</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>7937</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>2968625</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>142874</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="53" name="TextBox 52">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000035000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5770563" y="9080500"/>
-          <a:ext cx="1658937" cy="198437"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>23813</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>23812</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3016250</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>127000</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="54" name="TextBox 53">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000036000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4484688" y="9334500"/>
-          <a:ext cx="2992437" cy="103188"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>31752</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>31749</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3024189</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>134937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="55" name="TextBox 54">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000037000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4492627" y="9517062"/>
-          <a:ext cx="2992437" cy="103188"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>39689</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>23814</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032126</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>127002</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="56" name="TextBox 55">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000038000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4500564" y="9683752"/>
-          <a:ext cx="2992437" cy="103188"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="0"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>277813</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>912812</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>357188</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="57" name="TextBox 56">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000039000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="579438" y="9977438"/>
-          <a:ext cx="2992437" cy="214313"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>7937</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>142875</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3000374</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>357188</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="58" name="TextBox 57">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4468812" y="9977438"/>
-          <a:ext cx="2992437" cy="214313"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>246062</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>539749</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>134936</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="60" name="TextBox 59">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003C000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="301625" y="10787062"/>
-          <a:ext cx="539749" cy="134937"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1"/>
-            <a:t>2</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>539749</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>134937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="61" name="TextBox 60">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003D000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="301625" y="10961688"/>
-          <a:ext cx="539749" cy="134937"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>539749</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>134937</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="62" name="TextBox 61">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="301625" y="11136313"/>
-          <a:ext cx="539749" cy="134937"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032125</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>150812</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="63" name="TextBox 62">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00003F000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4460875" y="10787063"/>
-          <a:ext cx="3032125" cy="150812"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032125</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>150812</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="TextBox 63">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000040000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4460875" y="10961688"/>
-          <a:ext cx="3032125" cy="150812"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>3032125</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>150812</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="65" name="TextBox 64">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000041000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4460875" y="11136313"/>
-          <a:ext cx="3032125" cy="150812"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>754062</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>492125</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>785812</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>706438</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="66" name="TextBox 65">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000042000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2254250" y="11803063"/>
-          <a:ext cx="2992437" cy="214313"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>150813</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>47627</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>889000</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>317501</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="67" name="TextBox 66">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000043000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="277813" y="1936752"/>
-          <a:ext cx="2111375" cy="269874"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1"/>
-            <a:t>Human</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t> Resource Department</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
@@ -4970,7 +3080,7 @@
         <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33D97640-F776-0A02-DAD8-8F94FB819D6D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -5350,57 +3460,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="50"/>
+      <c r="A1" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="49"/>
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:14" s="2" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="55" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="N2" s="44"/>
+      <c r="A2" s="54" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="N2" s="43"/>
     </row>
     <row r="3" spans="1:14" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51"/>
       <c r="J3" s="1"/>
-      <c r="N3" s="44"/>
+      <c r="N3" s="43"/>
     </row>
     <row r="4" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
       <c r="D4" s="23"/>
       <c r="E4" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -5412,9 +3522,9 @@
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="64"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
+      <c r="B5" s="63"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
       <c r="E5" s="65"/>
       <c r="F5" s="65"/>
       <c r="G5" s="65"/>
@@ -5429,8 +3539,8 @@
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
-      <c r="E6" s="35" t="s">
-        <v>29</v>
+      <c r="E6" s="34" t="s">
+        <v>28</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -5449,30 +3559,30 @@
       <c r="I7" s="9"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:14" s="38" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="36"/>
-      <c r="B8" s="61" t="s">
+    <row r="8" spans="1:14" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="35"/>
+      <c r="B8" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="37"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="60"/>
+      <c r="I8" s="61"/>
+      <c r="J8" s="36"/>
     </row>
     <row r="9" spans="1:14" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
       <c r="F9" s="14"/>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="48" t="s">
         <v>18</v>
       </c>
       <c r="H9" s="13"/>
@@ -5494,15 +3604,15 @@
     <row r="11" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="2"/>
-      <c r="C11" s="47" t="s">
-        <v>50</v>
-      </c>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="48"/>
+      <c r="C11" s="46" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="47"/>
       <c r="G11" s="2"/>
       <c r="H11" s="29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I11" s="9"/>
       <c r="J11" s="1"/>
@@ -5511,10 +3621,10 @@
     <row r="12" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="2"/>
-      <c r="C12" s="47"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="48"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="47"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="9"/>
@@ -5523,15 +3633,15 @@
     <row r="13" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="8"/>
       <c r="B13" s="2"/>
-      <c r="C13" s="47" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="F13" s="48"/>
+      <c r="C13" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="46"/>
+      <c r="E13" s="46"/>
+      <c r="F13" s="47"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="48" t="s">
+      <c r="I13" s="47" t="s">
         <v>14</v>
       </c>
       <c r="J13" s="1"/>
@@ -5540,38 +3650,38 @@
     <row r="14" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="2"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="48"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="47"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="48"/>
+      <c r="I14" s="47"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="47" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="48"/>
+      <c r="C15" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="46"/>
+      <c r="E15" s="46"/>
+      <c r="F15" s="47"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="48" t="s">
-        <v>67</v>
+      <c r="I15" s="47" t="s">
+        <v>65</v>
       </c>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:14" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="48"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="46"/>
+      <c r="F16" s="47"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="9"/>
@@ -5580,12 +3690,12 @@
     <row r="17" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="47" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="47"/>
-      <c r="E17" s="47"/>
-      <c r="F17" s="48"/>
+      <c r="C17" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="46"/>
+      <c r="E17" s="46"/>
+      <c r="F17" s="47"/>
       <c r="G17" s="2"/>
       <c r="H17" s="29" t="s">
         <v>19</v>
@@ -5596,10 +3706,10 @@
     <row r="18" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="47"/>
-      <c r="D18" s="47"/>
-      <c r="E18" s="47"/>
-      <c r="F18" s="48"/>
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="46"/>
+      <c r="F18" s="47"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="9"/>
@@ -5607,43 +3717,43 @@
     </row>
     <row r="19" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
-      <c r="C19" s="47" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="48"/>
+      <c r="C19" s="46" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="47"/>
       <c r="G19" s="2"/>
-      <c r="H19" s="51"/>
-      <c r="I19" s="48" t="s">
-        <v>60</v>
+      <c r="H19" s="50"/>
+      <c r="I19" s="47" t="s">
+        <v>58</v>
       </c>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="48"/>
+      <c r="C20" s="46"/>
+      <c r="D20" s="46"/>
+      <c r="E20" s="46"/>
+      <c r="F20" s="47"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-      <c r="I20" s="48"/>
+      <c r="I20" s="47"/>
       <c r="J20" s="1"/>
     </row>
     <row r="21" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
-      <c r="C21" s="47" t="s">
-        <v>47</v>
-      </c>
-      <c r="D21" s="47"/>
-      <c r="E21" s="47"/>
-      <c r="F21" s="48"/>
+      <c r="C21" s="46" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="47"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="48" t="s">
-        <v>66</v>
+      <c r="I21" s="47" t="s">
+        <v>64</v>
       </c>
       <c r="J21" s="1"/>
       <c r="L21" s="2"/>
@@ -5652,10 +3762,10 @@
     <row r="22" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
-      <c r="E22" s="47"/>
-      <c r="F22" s="48"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="47"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="9"/>
@@ -5667,12 +3777,12 @@
     <row r="23" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="48"/>
+      <c r="C23" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="47"/>
       <c r="H23" s="2" t="s">
         <v>24</v>
       </c>
@@ -5682,10 +3792,10 @@
     <row r="24" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="48"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="47"/>
       <c r="G24" s="2"/>
       <c r="I24" s="27"/>
       <c r="J24" s="1"/>
@@ -5695,12 +3805,12 @@
     <row r="25" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="47" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="48"/>
+      <c r="C25" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="47"/>
       <c r="G25" s="2"/>
       <c r="H25" s="29" t="s">
         <v>22</v>
@@ -5713,10 +3823,10 @@
     <row r="26" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="48"/>
+      <c r="C26" s="46"/>
+      <c r="D26" s="46"/>
+      <c r="E26" s="46"/>
+      <c r="F26" s="47"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="27"/>
@@ -5728,15 +3838,15 @@
     <row r="27" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="8"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="47" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="48"/>
+      <c r="C27" s="46" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="46"/>
+      <c r="E27" s="46"/>
+      <c r="F27" s="47"/>
       <c r="G27" s="2"/>
       <c r="H27" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I27" s="27"/>
       <c r="J27" s="1"/>
@@ -5746,10 +3856,10 @@
     <row r="28" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="8"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="48"/>
+      <c r="C28" s="46"/>
+      <c r="D28" s="46"/>
+      <c r="E28" s="46"/>
+      <c r="F28" s="47"/>
       <c r="G28" s="2"/>
       <c r="I28" s="27"/>
       <c r="J28" s="1"/>
@@ -5760,12 +3870,12 @@
     <row r="29" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="8"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="47" t="s">
-        <v>48</v>
-      </c>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="48"/>
+      <c r="C29" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="47"/>
       <c r="G29" s="2"/>
       <c r="H29" t="s">
         <v>24</v>
@@ -5776,10 +3886,10 @@
     <row r="30" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="48"/>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="2"/>
       <c r="I30" s="27"/>
       <c r="J30" s="1"/>
@@ -5789,12 +3899,12 @@
     <row r="31" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="53" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="C31" s="52" t="s">
+        <v>55</v>
+      </c>
+      <c r="D31" s="52"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="53"/>
       <c r="G31" s="2"/>
       <c r="H31" s="29" t="s">
         <v>20</v>
@@ -5807,10 +3917,10 @@
     <row r="32" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="48"/>
+      <c r="C32" s="46"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="47"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="9"/>
@@ -5822,16 +3932,16 @@
     <row r="33" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="47" t="s">
-        <v>58</v>
-      </c>
-      <c r="D33" s="47"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="48"/>
+      <c r="C33" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="47"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="51"/>
-      <c r="I33" s="48" t="s">
-        <v>33</v>
+      <c r="H33" s="50"/>
+      <c r="I33" s="47" t="s">
+        <v>32</v>
       </c>
       <c r="J33" s="1"/>
       <c r="L33" s="2"/>
@@ -5846,21 +3956,21 @@
       <c r="F34" s="9"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="48"/>
+      <c r="I34" s="47"/>
       <c r="J34" s="1"/>
     </row>
     <row r="35" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="47" t="s">
-        <v>59</v>
+      <c r="C35" s="46" t="s">
+        <v>57</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
       <c r="F35" s="9"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="48" t="s">
+      <c r="I35" s="47" t="s">
         <v>21</v>
       </c>
       <c r="J35" s="1"/>
@@ -5868,7 +3978,7 @@
     <row r="36" spans="1:13" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="8"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="47"/>
+      <c r="C36" s="46"/>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="9"/>
@@ -5879,7 +3989,7 @@
     <row r="37" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="8"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="47"/>
+      <c r="C37" s="46"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="9"/>
@@ -5905,7 +4015,7 @@
     <row r="39" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="8"/>
       <c r="B39" s="29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -5913,7 +4023,7 @@
       <c r="F39" s="9"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
-      <c r="I39" s="48" t="s">
+      <c r="I39" s="47" t="s">
         <v>16</v>
       </c>
       <c r="J39" s="1"/>
@@ -5927,22 +4037,20 @@
       <c r="F40" s="9"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="48"/>
+      <c r="I40" s="47"/>
       <c r="J40" s="1"/>
     </row>
     <row r="41" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="8"/>
-      <c r="B41" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="B41" s="74"/>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
       <c r="E41" s="2"/>
       <c r="F41" s="9"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
-      <c r="I41" s="48" t="s">
-        <v>31</v>
+      <c r="I41" s="47" t="s">
+        <v>30</v>
       </c>
       <c r="J41" s="1"/>
     </row>
@@ -5968,7 +4076,7 @@
       <c r="E43" s="2"/>
       <c r="F43" s="9"/>
       <c r="G43" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I43" s="27"/>
       <c r="J43" s="1"/>
@@ -5986,16 +4094,14 @@
     </row>
     <row r="45" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
-      <c r="B45" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
+      <c r="B45" s="71"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
       <c r="E45" s="2"/>
       <c r="F45" s="9"/>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
-      <c r="I45" s="48" t="s">
+      <c r="I45" s="47" t="s">
         <v>2</v>
       </c>
       <c r="J45" s="1"/>
@@ -6009,7 +4115,7 @@
       <c r="F46" s="9"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
-      <c r="I46" s="48"/>
+      <c r="I46" s="47"/>
       <c r="J46" s="1"/>
     </row>
     <row r="47" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -6023,18 +4129,16 @@
       <c r="F47" s="9"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
-      <c r="I47" s="48" t="s">
+      <c r="I47" s="47" t="s">
         <v>3</v>
       </c>
       <c r="J47" s="1"/>
     </row>
     <row r="48" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
-      <c r="B48" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="C48" s="33"/>
-      <c r="D48" s="33"/>
+      <c r="B48" s="72"/>
+      <c r="C48" s="73"/>
+      <c r="D48" s="73"/>
       <c r="E48" s="33"/>
       <c r="F48" s="9"/>
       <c r="G48" s="1"/>
@@ -6049,26 +4153,26 @@
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="9"/>
-      <c r="G49" s="63" t="s">
+      <c r="G49" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="H49" s="59"/>
-      <c r="I49" s="60"/>
+      <c r="H49" s="58"/>
+      <c r="I49" s="59"/>
       <c r="J49" s="1"/>
     </row>
-    <row r="50" spans="1:10" s="38" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="36"/>
-      <c r="B50" s="61" t="s">
+    <row r="50" spans="1:10" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="35"/>
+      <c r="B50" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="61"/>
-      <c r="D50" s="61"/>
-      <c r="E50" s="61"/>
-      <c r="F50" s="61"/>
-      <c r="G50" s="61"/>
-      <c r="H50" s="61"/>
-      <c r="I50" s="62"/>
-      <c r="J50" s="37"/>
+      <c r="C50" s="60"/>
+      <c r="D50" s="60"/>
+      <c r="E50" s="60"/>
+      <c r="F50" s="60"/>
+      <c r="G50" s="60"/>
+      <c r="H50" s="60"/>
+      <c r="I50" s="61"/>
+      <c r="J50" s="36"/>
     </row>
     <row r="51" spans="1:10" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
@@ -6100,8 +4204,8 @@
     </row>
     <row r="53" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="8"/>
-      <c r="C53" s="45" t="s">
-        <v>42</v>
+      <c r="C53" s="44" t="s">
+        <v>41</v>
       </c>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
@@ -6130,24 +4234,24 @@
       <c r="B55" s="2"/>
       <c r="C55" s="15"/>
       <c r="D55" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E55" s="16" t="s">
         <v>36</v>
-      </c>
-      <c r="E55" s="16" t="s">
-        <v>37</v>
       </c>
       <c r="F55" s="9"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="9" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J55" s="1"/>
     </row>
     <row r="56" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="8"/>
       <c r="B56" s="2"/>
-      <c r="C56" s="46" t="s">
-        <v>38</v>
+      <c r="C56" s="45" t="s">
+        <v>37</v>
       </c>
       <c r="D56" s="17"/>
       <c r="E56" s="17"/>
@@ -6155,15 +4259,15 @@
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J56" s="1"/>
     </row>
     <row r="57" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="8"/>
       <c r="B57" s="2"/>
-      <c r="C57" s="46" t="s">
-        <v>39</v>
+      <c r="C57" s="45" t="s">
+        <v>38</v>
       </c>
       <c r="D57" s="17"/>
       <c r="E57" s="17"/>
@@ -6171,15 +4275,15 @@
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J57" s="1"/>
     </row>
     <row r="58" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="8"/>
       <c r="B58" s="2"/>
-      <c r="C58" s="46" t="s">
-        <v>40</v>
+      <c r="C58" s="45" t="s">
+        <v>39</v>
       </c>
       <c r="D58" s="17"/>
       <c r="E58" s="17"/>
@@ -6187,39 +4291,39 @@
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J58" s="1"/>
     </row>
     <row r="59" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="8"/>
       <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
+      <c r="C59" s="75"/>
+      <c r="D59" s="75"/>
+      <c r="E59" s="75"/>
       <c r="F59" s="2"/>
       <c r="G59" s="8"/>
       <c r="H59" s="2"/>
       <c r="I59" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J59" s="1"/>
     </row>
-    <row r="60" spans="1:10" s="43" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="39"/>
-      <c r="B60" s="40"/>
-      <c r="C60" s="57" t="s">
+    <row r="60" spans="1:10" s="42" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="38"/>
+      <c r="B60" s="39"/>
+      <c r="C60" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="57"/>
-      <c r="E60" s="57"/>
-      <c r="F60" s="41"/>
-      <c r="G60" s="58" t="s">
+      <c r="D60" s="56"/>
+      <c r="E60" s="56"/>
+      <c r="F60" s="40"/>
+      <c r="G60" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="H60" s="59"/>
-      <c r="I60" s="60"/>
-      <c r="J60" s="42"/>
+      <c r="H60" s="58"/>
+      <c r="I60" s="59"/>
+      <c r="J60" s="41"/>
     </row>
     <row r="61" spans="1:10" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
@@ -6241,14 +4345,14 @@
       <c r="A62" s="8"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="1"/>
       <c r="I62" s="11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J62" s="1"/>
     </row>
@@ -6256,14 +4360,14 @@
       <c r="A63" s="8"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J63" s="1"/>
     </row>
@@ -6271,20 +4375,20 @@
       <c r="A64" s="8"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J64" s="1"/>
     </row>
     <row r="65" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="67" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B65" s="68"/>
       <c r="C65" s="68"/>
@@ -6362,7 +4466,7 @@
       <c r="I71" s="70"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
     <mergeCell ref="A65:I65"/>
     <mergeCell ref="A67:I67"/>
     <mergeCell ref="A68:I68"/>
@@ -6380,6 +4484,7 @@
     <mergeCell ref="B50:I50"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:I5"/>
+    <mergeCell ref="C59:E59"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.5" right="0.5" top="0.25" bottom="0" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update HRIS workflows and UI
</commit_message>
<xml_diff>
--- a/leave application/CS Form No. 6, Revised 2020 (Application for Leave) (Fillable).xlsx
+++ b/leave application/CS Form No. 6, Revised 2020 (Application for Leave) (Fillable).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bless\Music\boac-personnel-hub\leave application\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\HRIS\leave application\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DDFB5F-8EF8-4A03-B2FA-3A15835B02B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE509B0B-F1A2-4779-A6CE-30440FC89686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -918,6 +918,28 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -966,28 +988,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3072,8 +3072,8 @@
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>455543</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>12565</xdr:rowOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>630048</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3104,6 +3104,56 @@
         <a:xfrm>
           <a:off x="1316935" y="497304"/>
           <a:ext cx="637760" cy="625131"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>998005</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>476250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>481691</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>671625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1293781" y="476250"/>
+          <a:ext cx="681831" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3460,45 +3510,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
       <c r="I1" s="49"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:14" s="2" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
+    <row r="2" spans="1:14" s="2" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="62" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="I2" s="54"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
       <c r="N2" s="43"/>
     </row>
     <row r="3" spans="1:14" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
       <c r="J3" s="1"/>
       <c r="N3" s="43"/>
     </row>
@@ -3522,14 +3572,14 @@
       <c r="A5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="63"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="66"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="72"/>
+      <c r="D5" s="72"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="74"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:14" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3561,16 +3611,16 @@
     </row>
     <row r="8" spans="1:14" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
-      <c r="G8" s="60"/>
-      <c r="H8" s="60"/>
-      <c r="I8" s="61"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="68"/>
+      <c r="I8" s="69"/>
       <c r="J8" s="36"/>
     </row>
     <row r="9" spans="1:14" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
@@ -3899,12 +3949,12 @@
     <row r="31" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="52" t="s">
+      <c r="C31" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="53"/>
+      <c r="D31" s="60"/>
+      <c r="E31" s="60"/>
+      <c r="F31" s="61"/>
       <c r="G31" s="2"/>
       <c r="H31" s="29" t="s">
         <v>20</v>
@@ -4042,7 +4092,7 @@
     </row>
     <row r="41" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="8"/>
-      <c r="B41" s="74"/>
+      <c r="B41" s="54"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" s="2"/>
@@ -4094,7 +4144,7 @@
     </row>
     <row r="45" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="8"/>
-      <c r="B45" s="71"/>
+      <c r="B45" s="51"/>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
       <c r="E45" s="2"/>
@@ -4136,9 +4186,9 @@
     </row>
     <row r="48" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="8"/>
-      <c r="B48" s="72"/>
-      <c r="C48" s="73"/>
-      <c r="D48" s="73"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="53"/>
+      <c r="D48" s="53"/>
       <c r="E48" s="33"/>
       <c r="F48" s="9"/>
       <c r="G48" s="1"/>
@@ -4153,25 +4203,25 @@
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="9"/>
-      <c r="G49" s="62" t="s">
+      <c r="G49" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="H49" s="58"/>
-      <c r="I49" s="59"/>
+      <c r="H49" s="66"/>
+      <c r="I49" s="67"/>
       <c r="J49" s="1"/>
     </row>
     <row r="50" spans="1:10" s="37" customFormat="1" ht="21.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A50" s="35"/>
-      <c r="B50" s="60" t="s">
+      <c r="B50" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="C50" s="60"/>
-      <c r="D50" s="60"/>
-      <c r="E50" s="60"/>
-      <c r="F50" s="60"/>
-      <c r="G50" s="60"/>
-      <c r="H50" s="60"/>
-      <c r="I50" s="61"/>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
+      <c r="E50" s="68"/>
+      <c r="F50" s="68"/>
+      <c r="G50" s="68"/>
+      <c r="H50" s="68"/>
+      <c r="I50" s="69"/>
       <c r="J50" s="36"/>
     </row>
     <row r="51" spans="1:10" ht="20.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
@@ -4312,17 +4362,17 @@
     <row r="60" spans="1:10" s="42" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="38"/>
       <c r="B60" s="39"/>
-      <c r="C60" s="56" t="s">
+      <c r="C60" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="56"/>
-      <c r="E60" s="56"/>
+      <c r="D60" s="64"/>
+      <c r="E60" s="64"/>
       <c r="F60" s="40"/>
-      <c r="G60" s="57" t="s">
+      <c r="G60" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="H60" s="58"/>
-      <c r="I60" s="59"/>
+      <c r="H60" s="66"/>
+      <c r="I60" s="67"/>
       <c r="J60" s="41"/>
     </row>
     <row r="61" spans="1:10" ht="19.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
@@ -4387,17 +4437,17 @@
       <c r="J64" s="1"/>
     </row>
     <row r="65" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="67" t="s">
+      <c r="A65" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="B65" s="68"/>
-      <c r="C65" s="68"/>
-      <c r="D65" s="68"/>
-      <c r="E65" s="68"/>
-      <c r="F65" s="68"/>
-      <c r="G65" s="68"/>
-      <c r="H65" s="68"/>
-      <c r="I65" s="69"/>
+      <c r="B65" s="56"/>
+      <c r="C65" s="56"/>
+      <c r="D65" s="56"/>
+      <c r="E65" s="56"/>
+      <c r="F65" s="56"/>
+      <c r="G65" s="56"/>
+      <c r="H65" s="56"/>
+      <c r="I65" s="57"/>
     </row>
     <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A66" s="30"/>
@@ -4411,68 +4461,62 @@
       <c r="I66" s="30"/>
     </row>
     <row r="67" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="70"/>
-      <c r="B67" s="70"/>
-      <c r="C67" s="70"/>
-      <c r="D67" s="70"/>
-      <c r="E67" s="70"/>
-      <c r="F67" s="70"/>
-      <c r="G67" s="70"/>
-      <c r="H67" s="70"/>
-      <c r="I67" s="70"/>
+      <c r="A67" s="58"/>
+      <c r="B67" s="58"/>
+      <c r="C67" s="58"/>
+      <c r="D67" s="58"/>
+      <c r="E67" s="58"/>
+      <c r="F67" s="58"/>
+      <c r="G67" s="58"/>
+      <c r="H67" s="58"/>
+      <c r="I67" s="58"/>
     </row>
     <row r="68" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="70"/>
-      <c r="B68" s="70"/>
-      <c r="C68" s="70"/>
-      <c r="D68" s="70"/>
-      <c r="E68" s="70"/>
-      <c r="F68" s="70"/>
-      <c r="G68" s="70"/>
-      <c r="H68" s="70"/>
-      <c r="I68" s="70"/>
+      <c r="A68" s="58"/>
+      <c r="B68" s="58"/>
+      <c r="C68" s="58"/>
+      <c r="D68" s="58"/>
+      <c r="E68" s="58"/>
+      <c r="F68" s="58"/>
+      <c r="G68" s="58"/>
+      <c r="H68" s="58"/>
+      <c r="I68" s="58"/>
     </row>
     <row r="69" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="70"/>
-      <c r="B69" s="70"/>
-      <c r="C69" s="70"/>
-      <c r="D69" s="70"/>
-      <c r="E69" s="70"/>
-      <c r="F69" s="70"/>
-      <c r="G69" s="70"/>
-      <c r="H69" s="70"/>
-      <c r="I69" s="70"/>
+      <c r="A69" s="58"/>
+      <c r="B69" s="58"/>
+      <c r="C69" s="58"/>
+      <c r="D69" s="58"/>
+      <c r="E69" s="58"/>
+      <c r="F69" s="58"/>
+      <c r="G69" s="58"/>
+      <c r="H69" s="58"/>
+      <c r="I69" s="58"/>
     </row>
     <row r="70" spans="1:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="70"/>
-      <c r="B70" s="70"/>
-      <c r="C70" s="70"/>
-      <c r="D70" s="70"/>
-      <c r="E70" s="70"/>
-      <c r="F70" s="70"/>
-      <c r="G70" s="70"/>
-      <c r="H70" s="70"/>
-      <c r="I70" s="70"/>
+      <c r="A70" s="58"/>
+      <c r="B70" s="58"/>
+      <c r="C70" s="58"/>
+      <c r="D70" s="58"/>
+      <c r="E70" s="58"/>
+      <c r="F70" s="58"/>
+      <c r="G70" s="58"/>
+      <c r="H70" s="58"/>
+      <c r="I70" s="58"/>
     </row>
     <row r="71" spans="1:9" s="28" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="70"/>
-      <c r="B71" s="70"/>
-      <c r="C71" s="70"/>
-      <c r="D71" s="70"/>
-      <c r="E71" s="70"/>
-      <c r="F71" s="70"/>
-      <c r="G71" s="70"/>
-      <c r="H71" s="70"/>
-      <c r="I71" s="70"/>
+      <c r="A71" s="58"/>
+      <c r="B71" s="58"/>
+      <c r="C71" s="58"/>
+      <c r="D71" s="58"/>
+      <c r="E71" s="58"/>
+      <c r="F71" s="58"/>
+      <c r="G71" s="58"/>
+      <c r="H71" s="58"/>
+      <c r="I71" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A65:I65"/>
-    <mergeCell ref="A67:I67"/>
-    <mergeCell ref="A68:I68"/>
-    <mergeCell ref="A69:I69"/>
-    <mergeCell ref="A71:I71"/>
-    <mergeCell ref="A70:I70"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="A2:I2"/>
@@ -4485,6 +4529,12 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:I5"/>
     <mergeCell ref="C59:E59"/>
+    <mergeCell ref="A65:I65"/>
+    <mergeCell ref="A67:I67"/>
+    <mergeCell ref="A68:I68"/>
+    <mergeCell ref="A69:I69"/>
+    <mergeCell ref="A71:I71"/>
+    <mergeCell ref="A70:I70"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.5" right="0.5" top="0.25" bottom="0" header="0.5" footer="0.5"/>

</xml_diff>